<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-05 La poire de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-05.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-05.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La poire dorée de Sarah</t>
+          <t>La poire de Sarah</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, poirier, panier de la voisine</t>
+          <t>marché, feuille jaune sur l'étal, vent, balance de fer, poires, torchon à carreaux, panier d'osier</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut la poire à joue dorée dans le panier sous le poirier. Elle dit bonjour, s'il te plaît, merci. Le jus reste froid.</t>
+          <t>Une feuille jaune tremble sur l'étal. Sur la poire, un éclat de poire brille. Sarah veut la poire maintenant. Elle tend la main trop vite, sans le mot : le doigt tape la balance. Elle refuse de foncer, dit s'il te plaît, obtient la poire. Merci vécu. Un éclat de poire reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les feuilles du poirier font une ombre ronde. Un panier d'osier attend au pied. Une poire a une joue dorée. Ça sent le sucré, tout près. L'herbe est chaude, un peu sèche. Un arrosoir de zinc sonne contre une pierre. Tu as vu la joue dorée, Sarah ? Elle brille, maman. C'est la poire du panier. La voisine remplit l'arrosoir. L'eau chante dans le zinc. Un oiseau picore sous l'arbre, tout petit. Il cherche une miette. Il n'en a pas. En ce moment, Sarah s'approche du panier. La poire courte est bien ronde. Sa peau est lisse, un peu froide. Celle-là, papa. On lui parle tout doux. L'arrosoir est encore plein. La voisine pose l'arrosoir près de la pierre. Elle se tourne vers le panier. Sarah se tient près de maman. Une petite feuille tient encore à la queue. Elle a un chapeau. Un tout petit chapeau. Tu demandes, Sarah.</t>
+          <t>Une feuille jaune tremble sur l'étal. Le vent la soulève, puis la repose. Une balance de fer fait tic. Elle fait tic, papa. Tu l'entends, Sarah ? Des caisses s'alignent sous le vent. Tu tiens ma manche, Sarah ? Un torchon à carreaux couvre une caisse. Le torchon claque un peu au vent. Maman tient un panier d'osier. L'osier gratte contre le manteau. Il pique un peu. C'est l'osier, près du bras. Le vent pousse la feuille. Elle est jaune. Un oiseau picore sous l'étal. Ça sent le sucré, près du nez. Ça sent bon, maman. Ce sont les poires. Les poires sont vertes, un côté doré. Sur la poire, un éclat de poire brille. Il brille, papa. Tu le vois, sur la peau ? Sarah touche l'éclat de poire. La peau est lisse, un peu froide. Elle est froide. Je la veux, maintenant ! Tu restes près de nous ? Oui, maman. Le fer de la balance est froid. Il est froid, le fer. Le vent pique un peu les joues. J'ai les joues froides. On avance. En ce moment, Sarah s'approche des poires. Une poire courte attend, bien ronde. Celle-là ! Sarah tend la main trop vite. Le doigt tape la balance de fer. Oh. La poire reste sur l'étal. La balance fait tic, puis se tait. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La poire est sur le bois. Tu la vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les feuilles du poirier font une ombre ronde. Un panier d'osier attend au pied. Une poire a une joue dorée. Ça sent le sucré, tout près. L'herbe est chaude, un peu sèche. Un arrosoir de zinc sonne contre une pierre. Tu as vu la joue dorée, Sarah ? Elle brille, maman. C'est la poire du panier. La voisine remplit l'arrosoir. L'eau chante dans le zinc. Un oiseau picore sous l'arbre, tout petit. Il cherche une miette. Il n'en a pas. En ce moment, Sarah s'approche du panier. La poire courte est bien ronde. Sa peau est lisse, un peu froide. Celle-là, papa. On lui parle tout doux. L'arrosoir est encore plein. La voisine pose l'arrosoir près de la pierre. Elle se tourne vers le panier. Sarah se tient près de maman. Une petite feuille tient encore à la queue. Elle a un chapeau. Un tout petit chapeau. Tu demandes, Sarah.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une feuille jaune tremble sur l'étal. Le vent la soulève, puis la repose. Une balance de fer fait tic. Elle fait tic, papa. Tu l'entends, Sarah ? Des caisses s'alignent sous le vent. Tu tiens ma manche, Sarah ? Un torchon à carreaux couvre une caisse. Le torchon claque un peu au vent. Maman tient un panier d'osier. L'osier gratte contre le manteau. Il pique un peu. C'est l'osier, près du bras. Le vent pousse la feuille. Elle est jaune. Un oiseau picore sous l'étal. Ça sent le sucré, près du nez. Ça sent bon, maman. Ce sont les poires. Les poires sont vertes, un côté doré. Sur la poire, un &lt;emphasis level="moderate"&gt;éclat de poire&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur la peau ? Sarah touche l'éclat de poire. La peau est lisse, un peu froide. Elle est froide. Je la veux, maintenant ! Tu restes près de nous ? Oui, maman. Le fer de la balance est froid. Il est froid, le fer. Le vent pique un peu les joues. J'ai les joues froides. On avance. En ce moment, Sarah s'approche des poires. Une poire courte attend, bien ronde. Celle-là ! Sarah tend la main trop vite. Le doigt tape la balance de fer. Oh. La poire reste sur l'étal. La balance fait tic, puis se tait. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La poire est sur le bois. Tu la vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Louise marche avec maman. Elles vont au marché. Les fruits brillent. La marchande sourit. Louise dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Maman dit : bonjour. Louise pointe une poire. Elle dit : s'il te plaît. La marchande tend la poire. Louise dit : merci. Maman dit : merci. Louise tient la poire. Elle est lisse. Ça sent le sucré. Maman serre sa main. Louise répète : bonjour. S'il te plaît. Merci. Les trois mots sont là.&lt;/slow&gt; [pause]</t>
+          <t>Une feuille jaune tremble sur l'étal. Le vent la soulève, puis la repose. Une balance de fer fait tic. Elle fait tic, papa. Tu l'entends, Sarah ? Des caisses s'alignent sous le vent. Tu tiens ma manche, Sarah ? Un torchon à carreaux couvre une caisse. Le torchon claque un peu au vent. Maman tient un panier d'osier. L'osier gratte contre le manteau. Il pique un peu. C'est l'osier, près du bras. Le vent pousse la feuille. Elle est jaune. Un oiseau picore sous l'étal. Ça sent le sucré, près du nez. Ça sent bon, maman. Ce sont les poires. Les poires sont vertes, un côté doré. Sur la poire, un &lt;emphasis&gt;éclat de poire&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur la peau ? Sarah touche l'éclat de poire. La peau est lisse, un peu froide. Elle est froide. Je la veux, maintenant ! Tu restes près de nous ? Oui, maman. Le fer de la balance est froid. Il est froid, le fer. Le vent pique un peu les joues. J'ai les joues froides. On avance. En ce moment, Sarah s'approche des poires. Une poire courte attend, bien ronde. Celle-là ! Sarah tend la main trop vite. Le doigt tape la balance de fer. Oh. La poire reste sur l'étal. La balance fait tic, puis se tait. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La poire est sur le bois. Tu la vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de poire</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,43 +1324,70 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_poire_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les feuilles du poirier font une ombre ronde.
-narrateur|Un panier d'osier attend au pied.
-narrateur|Une poire a une joue dorée.
-narrateur|Ça sent le sucré, tout près.
-narrateur|L'herbe est chaude, un peu sèche.
-narrateur|Un arrosoir de zinc sonne contre une pierre.
-maman|Tu as vu la joue dorée, Sarah ?
-enfant-f|Elle brille, maman.
-papa|C'est la poire du panier.
-narrateur|La voisine remplit l'arrosoir.
-narrateur|L'eau chante dans le zinc.
-narrateur|Un oiseau picore sous l'arbre, tout petit.
-papa|Il cherche une miette.
-enfant-f|Il n'en a pas.
-narrateur|En ce moment, Sarah s'approche du panier.
-narrateur|La poire courte est bien ronde.
-narrateur|Sa peau est lisse, un peu froide.
-enfant-f|Celle-là, papa.
-papa|On lui parle tout doux.
-maman|L'arrosoir est encore plein.
-narrateur|La voisine pose l'arrosoir près de la pierre.
-narrateur|Elle se tourne vers le panier.
-narrateur|Sarah se tient près de maman.
-narrateur|Une petite feuille tient encore à la queue.
-enfant-f|Elle a un chapeau.
-maman|Un tout petit chapeau.
-maman|Tu demandes, Sarah.</t>
+          <t>narrateur|Une feuille jaune tremble sur l'étal.
+narrateur|Le vent la soulève, puis la repose.
+narrateur|Une balance de fer fait tic.
+enfant-f|Elle fait tic, papa.
+papa|Tu l'entends, Sarah ?
+narrateur|Des caisses s'alignent sous le vent.
+papa|Tu tiens ma manche, Sarah ?
+narrateur|Un torchon à carreaux couvre une caisse.
+narrateur|Le torchon claque un peu au vent.
+narrateur|Maman tient un panier d'osier.
+narrateur|L'osier gratte contre le manteau.
+enfant-f|Il pique un peu.
+maman|C'est l'osier, près du bras.
+papa|Le vent pousse la feuille.
+enfant-f|Elle est jaune.
+narrateur|Un oiseau picore sous l'étal.
+narrateur|Ça sent le sucré, près du nez.
+enfant-f|Ça sent bon, maman.
+maman|Ce sont les poires.
+narrateur|Les poires sont vertes, un côté doré.
+narrateur|Sur la poire, un éclat de poire brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, sur la peau ?
+narrateur|Sarah touche l'éclat de poire.
+narrateur|La peau est lisse, un peu froide.
+enfant-f|Elle est froide.
+enfant-f|Je la veux, maintenant !
+maman|Tu restes près de nous ?
+enfant-f|Oui, maman.
+papa|Le fer de la balance est froid.
+enfant-f|Il est froid, le fer.
+narrateur|Le vent pique un peu les joues.
+enfant-f|J'ai les joues froides.
+papa|On avance.
+narrateur|En ce moment, Sarah s'approche des poires.
+narrateur|Une poire courte attend, bien ronde.
+enfant-f|Celle-là !
+narrateur|Sarah tend la main trop vite.
+narrateur|Le doigt tape la balance de fer.
+enfant-f|Oh.
+narrateur|La poire reste sur l'étal.
+narrateur|La balance fait tic, puis se tait.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je la prends !
+maman|La poire est sur le bois.
+papa|Tu la vois, Sarah ?
+narrateur|Les épaules de Sarah tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>feuilles,eau</t>
+          <t>vent,balance</t>
         </is>
       </c>
     </row>
@@ -1392,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah veut la poire. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah veut la &lt;emphasis level="moderate"&gt;poire&lt;/emphasis&gt;. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Louise veut la poire. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah veut la &lt;emphasis&gt;poire&lt;/emphasis&gt;. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1460,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1468,10 +1495,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1486,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>poire</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1522,13 +1553,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1538,7 +1569,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_dit_s_il_te_plait; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1571,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une poire, s'il te plaît. Celle avec la joue. La voisine pose la poire. Elle est dans le panier d'osier. L'osier craque un tout petit peu. Merci. Merci. Sarah touche la poire du bout du doigt. Elle est lisse. Elle sent le sucré. Elle est froide, maman. Oui. Elle était sous les feuilles. Le chapeau est encore là. Tout petit. Sarah tient une anse du panier. Le panier penche un peu, tout doux. On rentre par l'herbe ? Oui, maman. L'oiseau n'est plus sous l'arbre.</t>
+          <t>Sarah avance trop vite vers l'étal. Celle-là, maintenant ! Sa voix se mélange au vent. Oh. La poire reste sur le bois. Elle refuse de foncer. Sarah referme la main. Elle écoute la balance, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Sarah pose un pied près de l'étal. Le bois est lisse, un peu froid. Celle-là. S'il te plaît. Derrière l'étal, une main se tend. La poire glisse dans le panier. L'osier craque contre la poire. Merci, Sarah. Papa a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le sucré et le bois. La poire est à moi. Elle est dans le panier. Sarah pose une main sur la poire. La peau est un peu froide. La balance se tait.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une poire, s'il te plaît. Celle avec la joue. La voisine pose la poire. Elle est dans le panier d'osier. L'osier craque un tout petit peu. Merci. Merci. Sarah touche la poire du bout du doigt. Elle est lisse. Elle sent le sucré. Elle est froide, maman. Oui. Elle était sous les feuilles. Le chapeau est encore là. Tout petit. Sarah tient une anse du panier. Le panier penche un peu, tout doux. On rentre par l'herbe ? Oui, maman. L'oiseau n'est plus sous l'arbre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah avance trop vite vers l'étal. Celle-là, maintenant ! Sa voix se mélange au vent. Oh. La poire reste sur le bois. Elle refuse de foncer. Sarah referme la main. Elle écoute la balance, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Sarah pose un pied près de l'étal. Le bois est lisse, un peu froid. Celle-là. &lt;emphasis level="moderate"&gt;S'il te plaît&lt;/emphasis&gt;. Derrière l'étal, une main se tend. La poire glisse dans le panier. L'osier craque contre la poire. Merci, Sarah. Papa a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le sucré et le bois. La poire est à moi. Elle est dans le panier. Sarah pose une main sur la poire. La peau est un peu froide. La balance se tait.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Louise a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Elle a dit s'il te plaît. Elle a dit merci. Maman est là.&lt;/slow&gt; [pause]</t>
+          <t>Sarah avance trop vite vers l'étal. Celle-là, maintenant ! Sa voix se mélange au vent. Oh. La poire reste sur le bois. Elle refuse de foncer. Sarah referme la main. Elle écoute la balance, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Sarah pose un pied près de l'étal. Le bois est lisse, un peu froid. Celle-là. &lt;emphasis&gt;S'il te plaît&lt;/emphasis&gt;. Derrière l'étal, une main se tend. La poire glisse dans le panier. L'osier craque contre la poire. Merci, Sarah. Papa a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le sucré et le bois. La poire est à moi. Elle est dans le panier. Sarah pose une main sur la poire. La peau est un peu froide. La balance se tait. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1628,18 +1659,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1662,7 +1693,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>S'il te plaît</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1672,20 +1703,20 @@
         <v>450</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1694,10 +1725,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1706,42 +1737,49 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_balance_echoue_le_mot_ouvre; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Bonjour.
-maman|Bonjour.
-enfant-f|Une poire, s'il te plaît.
-enfant-f|Celle avec la joue.
-narrateur|La voisine pose la poire.
-narrateur|Elle est dans le panier d'osier.
-narrateur|L'osier craque un tout petit peu.
-enfant-f|Merci.
-papa|Merci.
-narrateur|Sarah touche la poire du bout du doigt.
-narrateur|Elle est lisse.
-narrateur|Elle sent le sucré.
-enfant-f|Elle est froide, maman.
-maman|Oui.
-maman|Elle était sous les feuilles.
-papa|Le chapeau est encore là.
-enfant-f|Tout petit.
-narrateur|Sarah tient une anse du panier.
-narrateur|Le panier penche un peu, tout doux.
-maman|On rentre par l'herbe ?
-enfant-f|Oui, maman.
-narrateur|L'oiseau n'est plus sous l'arbre.</t>
+          <t>narrateur|Sarah avance trop vite vers l'étal.
+enfant-f|Celle-là, maintenant !
+narrateur|Sa voix se mélange au vent.
+enfant-f|Oh.
+narrateur|La poire reste sur le bois.
+narrateur|Elle refuse de foncer.
+narrateur|Sarah referme la main.
+narrateur|Elle écoute la balance, un instant.
+papa|Tu veux venir près du bois ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Sarah pose un pied près de l'étal.
+narrateur|Le bois est lisse, un peu froid.
+enfant-f|Celle-là.
+enfant-f|S'il te plaît.
+narrateur|Derrière l'étal, une main se tend.
+narrateur|La poire glisse dans le panier.
+narrateur|L'osier craque contre la poire.
+papa|Merci, Sarah.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Sarah se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-f|Un peu, maman.
+narrateur|Ça sent le sucré et le bois.
+enfant-f|La poire est à moi.
+maman|Elle est dans le panier.
+narrateur|Sarah pose une main sur la poire.
+narrateur|La peau est un peu froide.
+narrateur|La balance se tait.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>panier</t>
+          <t>panier,osier</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1806,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent le long de l'herbe sèche. Les feuilles du poirier bougent un peu. À la maison, maman pose le panier. Sarah prend la poire à deux mains. Tu veux un bout ? Oui, papa. S'il te plaît. Sarah croque. Le jus est sucré, un peu froid. Merci, papa. Merci, Sarah. La petite feuille reste sur la table. Son chapeau. Oui. On la met près de la fenêtre. Elle brille encore. Moins qu'au jardin. L'ombre du poirier n'est plus là. Le panier d'osier est vide, maintenant.</t>
+          <t>Sarah tire la poire trop vite. Je la mange, d'un coup ! La poire glisse dans l'osier. Elle penche vers le sol. Oh. Sarah avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Sarah observe l'étal, écoute le vent. Sur la peau, un éclat de poire luit. Là, près de la feuille. Sarah tient la poire des deux mains. La peau est lisse, un peu froide. Elle est froide, papa. Tu la portes jusqu'à la rue ? Oui, papa. On avance ? Oui, maman. Le vent reprend la feuille jaune. La feuille s'envole vers la rue. L'air froid revient sur les joues. Sarah serre la poire contre elle. Elle reste froide. On marche. La poire penche, puis se cale. Je la tiens. On avance. Sarah passe le long de l'étal. Le bois craque, un peu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent le long de l'herbe sèche. Les feuilles du poirier bougent un peu. À la maison, maman pose le panier. Sarah prend la poire à deux mains. Tu veux un bout ? Oui, papa. S'il te plaît. Sarah croque. Le jus est sucré, un peu froid. Merci, papa. Merci, Sarah. La petite feuille reste sur la table. Son chapeau. Oui. On la met près de la fenêtre. Elle brille encore. Moins qu'au jardin. L'ombre du poirier n'est plus là. Le panier d'osier est vide, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah tire la poire trop vite. Je la mange, d'un coup ! La poire glisse dans l'osier. Elle penche vers le sol. Oh. Sarah avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Sarah observe l'étal, écoute le vent. Sur la peau, un &lt;emphasis level="moderate"&gt;éclat de poire&lt;/emphasis&gt; luit. Là, près de la feuille. Sarah tient la poire des deux mains. La peau est lisse, un peu froide. Elle est froide, papa. Tu la portes jusqu'à la rue ? Oui, papa. On avance ? Oui, maman. Le vent reprend la feuille jaune. La feuille s'envole vers la rue. L'air froid revient sur les joues. Sarah serre la poire contre elle. Elle reste froide. On marche. La poire penche, puis se cale. Je la tiens. On avance. Sarah passe le long de l'étal. Le bois craque, un peu.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Louise croque un bout de poire. Maman sourit.&lt;/slow&gt; [pause]</t>
+          <t>Sarah tire la poire trop vite. Je la mange, d'un coup ! La poire glisse dans l'osier. Elle penche vers le sol. Oh. Sarah avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Sarah observe l'étal, écoute le vent. Sur la peau, un &lt;emphasis&gt;éclat de poire&lt;/emphasis&gt; luit. Là, près de la feuille. Sarah tient la poire des deux mains. La peau est lisse, un peu froide. Elle est froide, papa. Tu la portes jusqu'à la rue ? Oui, papa. On avance ? Oui, maman. Le vent reprend la feuille jaune. La feuille s'envole vers la rue. L'air froid revient sur les joues. Sarah serre la poire contre elle. Elle reste froide. On marche. La poire penche, puis se cale. Je la tiens. On avance. Sarah passe le long de l'étal. Le bois craque, un peu. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1825,18 +1863,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1857,28 +1895,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de poire</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1887,10 +1929,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1899,35 +1941,50 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils rentrent le long de l'herbe sèche.
-narrateur|Les feuilles du poirier bougent un peu.
-narrateur|À la maison, maman pose le panier.
-narrateur|Sarah prend la poire à deux mains.
-papa|Tu veux un bout ?
+          <t>narrateur|Sarah tire la poire trop vite.
+enfant-f|Je la mange, d'un coup !
+narrateur|La poire glisse dans l'osier.
+narrateur|Elle penche vers le sol.
+enfant-f|Oh.
+narrateur|Sarah avance les mains.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Sarah observe l'étal, écoute le vent.
+narrateur|Sur la peau, un éclat de poire luit.
+enfant-f|Là, près de la feuille.
+narrateur|Sarah tient la poire des deux mains.
+narrateur|La peau est lisse, un peu froide.
+enfant-f|Elle est froide, papa.
+papa|Tu la portes jusqu'à la rue ?
 enfant-f|Oui, papa.
-enfant-f|S'il te plaît.
-narrateur|Sarah croque.
-narrateur|Le jus est sucré, un peu froid.
-enfant-f|Merci, papa.
-maman|Merci, Sarah.
-narrateur|La petite feuille reste sur la table.
-papa|Son chapeau.
-enfant-f|Oui.
-maman|On la met près de la fenêtre.
-enfant-f|Elle brille encore.
-papa|Moins qu'au jardin.
-narrateur|L'ombre du poirier n'est plus là.
-narrateur|Le panier d'osier est vide, maintenant.</t>
+maman|On avance ?
+enfant-f|Oui, maman.
+narrateur|Le vent reprend la feuille jaune.
+narrateur|La feuille s'envole vers la rue.
+narrateur|L'air froid revient sur les joues.
+narrateur|Sarah serre la poire contre elle.
+enfant-f|Elle reste froide.
+papa|On marche.
+narrateur|La poire penche, puis se cale.
+enfant-f|Je la tiens.
+maman|On avance.
+narrateur|Sarah passe le long de l'étal.
+narrateur|Le bois craque, un peu.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>croque</t>
+          <t>vent,panier</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2011,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Il reste un bout, encore froid. La feuille dort près de la fenêtre. Bonne après-midi, Sarah. Elle avait une joue dorée.</t>
+          <t>La feuille brillait, papa. Tu la vois, comme sur l'étal ? Oui, dans le vent. Sarah pose la poire contre le manteau. On la garde au frais ? Oui, maman. L'étal sentait bon. Il est derrière nous. Une feuille jaune n'est plus là. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. La poire reste froide sous la main. Un éclat de poire reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Il reste un bout, encore froid. La feuille dort près de la fenêtre. Bonne après-midi, Sarah. Elle avait une joue dorée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La feuille brillait, papa. Tu la vois, comme sur l'étal ? Oui, dans le vent. Sarah pose la poire contre le manteau. On la garde au frais ? Oui, maman. L'étal sentait bon. Il est derrière nous. Une feuille jaune n'est plus là. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. La poire reste froide sous la main. Un &lt;emphasis level="moderate"&gt;éclat de poire&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La feuille brillait, papa. Tu la vois, comme sur l'étal ? Oui, dans le vent. Sarah pose la poire contre le manteau. On la garde au frais ? Oui, maman. L'étal sentait bon. Il est derrière nous. Une feuille jaune n'est plus là. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. La poire reste froide sous la main. Un &lt;emphasis&gt;éclat de poire&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,7 +2068,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2019,10 +2076,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2088,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2102,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de poire</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2125,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,27 +2138,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Il reste un bout, encore froid.
-narrateur|La feuille dort près de la fenêtre.
-maman|Bonne après-midi, Sarah.
-papa|Elle avait une joue dorée.</t>
+          <t>enfant-f|La feuille brillait, papa.
+papa|Tu la vois, comme sur l'étal ?
+enfant-f|Oui, dans le vent.
+narrateur|Sarah pose la poire contre le manteau.
+maman|On la garde au frais ?
+enfant-f|Oui, maman.
+enfant-f|L'étal sentait bon.
+maman|Il est derrière nous.
+narrateur|Une feuille jaune n'est plus là.
+narrateur|Sarah respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Sarah se réchauffent.
+narrateur|La poire reste froide sous la main.
+narrateur|Un éclat de poire reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>vent</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2210,6 +2291,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>